<commit_message>
Update and Fix Fitur
</commit_message>
<xml_diff>
--- a/Robot Monitoring.xlsx
+++ b/Robot Monitoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\xampp\htdocs\robot_dashboard\robot-navigasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323239A6-7E4A-44E3-BF68-4B56234ACA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9B39D1-B592-4420-BD2A-650409B07B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -403,9 +403,6 @@
     <t>Tertunda</t>
   </si>
   <si>
-    <t>Sedang Dikerjakan</t>
-  </si>
-  <si>
     <t>Diimplementasikan di sensors.php dengan monitoring real-time, tampilan persentase, volume dalam ml, dan indikator status</t>
   </si>
   <si>
@@ -424,9 +421,6 @@
     <t>Pelacakan posisi 3D (X, Y, Z) real-time di sensors.php</t>
   </si>
   <si>
-    <t>Belum diimplementasikan - memerlukan sensor tambahan</t>
-  </si>
-  <si>
     <t>Grafik dan tampilan numerik di index.php dan sensors.php menggunakan Chart.js</t>
   </si>
   <si>
@@ -442,9 +436,6 @@
     <t>Sistem logbook lengkap di logbook.php dengan filtering, export, dan logging real-time</t>
   </si>
   <si>
-    <t>Tahap Perencanaan mendefinisikan langkah-langkah yang diperlukan untuk memastikan perencanaan yang tepat dilakukan, selama memulai proyek, sebelum setiap fase baru dimulai dan sebagai bagian dari proses manajemen perubahan</t>
-  </si>
-  <si>
     <t>Diimplementasikan melalui Firebase Realtime Database</t>
   </si>
   <si>
@@ -454,9 +445,6 @@
     <t>Data real-time melalui Firebase listeners</t>
   </si>
   <si>
-    <t>Menetapkan Ruang Lingkup Proyek, WBS dan Deliverables yang diperlukan untuk memastikan bahwa tujuan yang didefinisikan dalam Project Charter terpenuhi.</t>
-  </si>
-  <si>
     <t>Dashboard multi-halaman: index.php, sensors.php, logbook.php</t>
   </si>
   <si>
@@ -472,9 +460,6 @@
     <t>Data historis di grafik dan logbook</t>
   </si>
   <si>
-    <t>Sebagian - konfigurasi Firebase tersedia</t>
-  </si>
-  <si>
     <t>Belum diimplementasikan - memerlukan integrasi ML</t>
   </si>
   <si>
@@ -484,21 +469,6 @@
     <t>Fungsi export CSV di logbook</t>
   </si>
   <si>
-    <t>Mengkoordinasikan orang dan sumber daya lain yang diperlukan untuk menyelesaikan proyek</t>
-  </si>
-  <si>
-    <t>Belum diimplementasikan - memerlukan sistem autentikasi</t>
-  </si>
-  <si>
-    <t>Sebagian - notifikasi browser melalui alert logbook</t>
-  </si>
-  <si>
-    <t>Sebagian - indikator visual untuk baterai rendah</t>
-  </si>
-  <si>
-    <t>Sebagian - logbook menangkap event</t>
-  </si>
-  <si>
     <t>Pelacakan GPS real-time di peta di index.php</t>
   </si>
   <si>
@@ -512,12 +482,45 @@
   </si>
   <si>
     <t>Palet warna konsisten dengan mode gelap/terang, ukuran dan spasi yang tepat</t>
+  </si>
+  <si>
+    <t>Semua komunikasi data real-time melalui Firebase Realtime Database sudah berjalan sempurna</t>
+  </si>
+  <si>
+    <t>Dashboard monitoring, visualisasi data, grafik real-time, logging, dan export data sudah lengkap</t>
+  </si>
+  <si>
+    <t>Sistem RBAC lengkap dengan autentikasi, authorization, session management, dan permission-based UI di auth.php</t>
+  </si>
+  <si>
+    <t>Sistem autentikasi lengkap dengan login, logout, session timeout, dan role-based authorization</t>
+  </si>
+  <si>
+    <t>Obstacle detection system dengan visualisasi di minimap, collision detection, auto-stop, dan obstacle editor</t>
+  </si>
+  <si>
+    <t>Konfigurasi Firebase, sistem multi-kamera, mode operasi, dan obstacle management sudah lengkap</t>
+  </si>
+  <si>
+    <t>Semua fitur kontrol, monitoring, RBAC, notifikasi, dan collision avoidance sudah diimplementasikan</t>
+  </si>
+  <si>
+    <t>Notifikasi browser, SweetAlert2, logbook real-time, alert visual, dan collision warnings sudah lengkap</t>
+  </si>
+  <si>
+    <t>Threshold monitoring untuk baterai, level cairan, sensor, dan proximity warning untuk obstacle</t>
+  </si>
+  <si>
+    <t>Logbook menangkap semua event termasuk collision detection, proximity alerts, dan obstacle events</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ hh:mm"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -547,8 +550,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -885,6 +890,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X51"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="15.125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -906,7 +915,7 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>46148.375</v>
       </c>
     </row>
@@ -914,7 +923,7 @@
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>46156.708333333299</v>
       </c>
     </row>
@@ -930,8 +939,8 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6">
-        <v>85</v>
+      <c r="B6" s="2">
+        <v>0.95</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
@@ -1043,20 +1052,20 @@
       <c r="G10" t="s">
         <v>11</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J10" t="s">
         <v>11</v>
       </c>
-      <c r="K10">
-        <v>90</v>
+      <c r="K10" s="2">
+        <v>1</v>
       </c>
       <c r="L10" t="s">
-        <v>11</v>
+        <v>125</v>
       </c>
       <c r="M10" t="s">
         <v>11</v>
@@ -1077,7 +1086,7 @@
         <v>38</v>
       </c>
       <c r="S10" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T10" t="s">
         <v>11</v>
@@ -1117,17 +1126,17 @@
       <c r="G11" t="s">
         <v>11</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J11" t="s">
         <v>11</v>
       </c>
-      <c r="K11">
-        <v>100</v>
+      <c r="K11" s="2">
+        <v>1</v>
       </c>
       <c r="L11" t="s">
         <v>125</v>
@@ -1148,7 +1157,7 @@
         <v>37</v>
       </c>
       <c r="R11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="S11" t="s">
         <v>42</v>
@@ -1197,8 +1206,8 @@
       <c r="J12" t="s">
         <v>11</v>
       </c>
-      <c r="K12">
-        <v>100</v>
+      <c r="K12" s="2">
+        <v>1</v>
       </c>
       <c r="L12" t="s">
         <v>125</v>
@@ -1219,7 +1228,7 @@
         <v>37</v>
       </c>
       <c r="R12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="S12" t="s">
         <v>42</v>
@@ -1262,17 +1271,17 @@
       <c r="G13" t="s">
         <v>11</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J13" t="s">
         <v>11</v>
       </c>
-      <c r="K13">
-        <v>100</v>
+      <c r="K13" s="2">
+        <v>1</v>
       </c>
       <c r="L13" t="s">
         <v>125</v>
@@ -1293,7 +1302,7 @@
         <v>37</v>
       </c>
       <c r="R13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="S13" t="s">
         <v>42</v>
@@ -1336,17 +1345,17 @@
       <c r="G14" t="s">
         <v>11</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J14" t="s">
         <v>11</v>
       </c>
-      <c r="K14">
-        <v>100</v>
+      <c r="K14" s="2">
+        <v>1</v>
       </c>
       <c r="L14" t="s">
         <v>125</v>
@@ -1367,7 +1376,7 @@
         <v>37</v>
       </c>
       <c r="R14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="S14" t="s">
         <v>42</v>
@@ -1410,17 +1419,17 @@
       <c r="G15" t="s">
         <v>11</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J15" t="s">
         <v>11</v>
       </c>
-      <c r="K15">
-        <v>100</v>
+      <c r="K15" s="2">
+        <v>1</v>
       </c>
       <c r="L15" t="s">
         <v>125</v>
@@ -1441,7 +1450,7 @@
         <v>37</v>
       </c>
       <c r="R15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="S15" t="s">
         <v>42</v>
@@ -1484,17 +1493,17 @@
       <c r="G16" t="s">
         <v>11</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J16" t="s">
         <v>11</v>
       </c>
-      <c r="K16">
-        <v>100</v>
+      <c r="K16" s="2">
+        <v>1</v>
       </c>
       <c r="L16" t="s">
         <v>125</v>
@@ -1515,7 +1524,7 @@
         <v>37</v>
       </c>
       <c r="R16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="S16" t="s">
         <v>42</v>
@@ -1558,20 +1567,20 @@
       <c r="G17" t="s">
         <v>11</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J17" t="s">
         <v>11</v>
       </c>
-      <c r="K17">
-        <v>0</v>
+      <c r="K17" s="2">
+        <v>1</v>
       </c>
       <c r="L17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M17" t="s">
         <v>11</v>
@@ -1589,10 +1598,10 @@
         <v>37</v>
       </c>
       <c r="R17" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="S17" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T17" t="s">
         <v>11</v>
@@ -1632,17 +1641,17 @@
       <c r="G18" t="s">
         <v>11</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J18" t="s">
         <v>11</v>
       </c>
-      <c r="K18">
-        <v>100</v>
+      <c r="K18" s="2">
+        <v>1</v>
       </c>
       <c r="L18" t="s">
         <v>125</v>
@@ -1663,7 +1672,7 @@
         <v>37</v>
       </c>
       <c r="R18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="S18" t="s">
         <v>42</v>
@@ -1706,17 +1715,17 @@
       <c r="G19" t="s">
         <v>11</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J19" t="s">
         <v>11</v>
       </c>
-      <c r="K19">
-        <v>100</v>
+      <c r="K19" s="2">
+        <v>1</v>
       </c>
       <c r="L19" t="s">
         <v>125</v>
@@ -1737,7 +1746,7 @@
         <v>37</v>
       </c>
       <c r="R19" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="S19" t="s">
         <v>42</v>
@@ -1780,17 +1789,17 @@
       <c r="G20" t="s">
         <v>11</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J20" t="s">
         <v>11</v>
       </c>
-      <c r="K20">
-        <v>100</v>
+      <c r="K20" s="2">
+        <v>1</v>
       </c>
       <c r="L20" t="s">
         <v>125</v>
@@ -1811,7 +1820,7 @@
         <v>37</v>
       </c>
       <c r="R20" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="S20" t="s">
         <v>42</v>
@@ -1854,17 +1863,17 @@
       <c r="G21" t="s">
         <v>11</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J21" t="s">
         <v>11</v>
       </c>
-      <c r="K21">
-        <v>100</v>
+      <c r="K21" s="2">
+        <v>1</v>
       </c>
       <c r="L21" t="s">
         <v>125</v>
@@ -1885,7 +1894,7 @@
         <v>37</v>
       </c>
       <c r="R21" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="S21" t="s">
         <v>42</v>
@@ -1928,17 +1937,17 @@
       <c r="G22" t="s">
         <v>11</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="1">
         <v>46149.375</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="1">
         <v>46156.708333333299</v>
       </c>
       <c r="J22" t="s">
         <v>11</v>
       </c>
-      <c r="K22">
-        <v>100</v>
+      <c r="K22" s="2">
+        <v>1</v>
       </c>
       <c r="L22" t="s">
         <v>125</v>
@@ -1959,7 +1968,7 @@
         <v>37</v>
       </c>
       <c r="R22" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="S22" t="s">
         <v>42</v>
@@ -2011,11 +2020,11 @@
       <c r="J23" t="s">
         <v>11</v>
       </c>
-      <c r="K23">
-        <v>80</v>
+      <c r="K23" s="2">
+        <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>11</v>
+        <v>125</v>
       </c>
       <c r="M23" t="s">
         <v>11</v>
@@ -2033,10 +2042,10 @@
         <v>42</v>
       </c>
       <c r="R23" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="S23" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T23" t="s">
         <v>11</v>
@@ -2085,8 +2094,8 @@
       <c r="J24" t="s">
         <v>11</v>
       </c>
-      <c r="K24">
-        <v>100</v>
+      <c r="K24" s="2">
+        <v>1</v>
       </c>
       <c r="L24" t="s">
         <v>125</v>
@@ -2107,7 +2116,7 @@
         <v>37</v>
       </c>
       <c r="R24" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="S24" t="s">
         <v>42</v>
@@ -2159,8 +2168,8 @@
       <c r="J25" t="s">
         <v>11</v>
       </c>
-      <c r="K25">
-        <v>100</v>
+      <c r="K25" s="2">
+        <v>1</v>
       </c>
       <c r="L25" t="s">
         <v>125</v>
@@ -2181,7 +2190,7 @@
         <v>37</v>
       </c>
       <c r="R25" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="S25" t="s">
         <v>42</v>
@@ -2233,8 +2242,8 @@
       <c r="J26" t="s">
         <v>11</v>
       </c>
-      <c r="K26">
-        <v>100</v>
+      <c r="K26" s="2">
+        <v>1</v>
       </c>
       <c r="L26" t="s">
         <v>125</v>
@@ -2255,7 +2264,7 @@
         <v>37</v>
       </c>
       <c r="R26" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="S26" t="s">
         <v>42</v>
@@ -2307,8 +2316,8 @@
       <c r="J27" t="s">
         <v>11</v>
       </c>
-      <c r="K27">
-        <v>100</v>
+      <c r="K27" s="2">
+        <v>1</v>
       </c>
       <c r="L27" t="s">
         <v>125</v>
@@ -2329,7 +2338,7 @@
         <v>37</v>
       </c>
       <c r="R27" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="S27" t="s">
         <v>42</v>
@@ -2381,11 +2390,11 @@
       <c r="J28" t="s">
         <v>11</v>
       </c>
-      <c r="K28">
-        <v>85</v>
+      <c r="K28" s="2">
+        <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>11</v>
+        <v>125</v>
       </c>
       <c r="M28" t="s">
         <v>11</v>
@@ -2403,10 +2412,10 @@
         <v>42</v>
       </c>
       <c r="R28" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="S28" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T28" t="s">
         <v>11</v>
@@ -2455,8 +2464,8 @@
       <c r="J29" t="s">
         <v>11</v>
       </c>
-      <c r="K29">
-        <v>100</v>
+      <c r="K29" s="2">
+        <v>1</v>
       </c>
       <c r="L29" t="s">
         <v>125</v>
@@ -2477,7 +2486,7 @@
         <v>37</v>
       </c>
       <c r="R29" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="S29" t="s">
         <v>42</v>
@@ -2529,8 +2538,8 @@
       <c r="J30" t="s">
         <v>11</v>
       </c>
-      <c r="K30">
-        <v>100</v>
+      <c r="K30" s="2">
+        <v>1</v>
       </c>
       <c r="L30" t="s">
         <v>125</v>
@@ -2551,7 +2560,7 @@
         <v>37</v>
       </c>
       <c r="R30" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="S30" t="s">
         <v>42</v>
@@ -2603,8 +2612,8 @@
       <c r="J31" t="s">
         <v>11</v>
       </c>
-      <c r="K31">
-        <v>100</v>
+      <c r="K31" s="2">
+        <v>1</v>
       </c>
       <c r="L31" t="s">
         <v>125</v>
@@ -2625,7 +2634,7 @@
         <v>37</v>
       </c>
       <c r="R31" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="S31" t="s">
         <v>42</v>
@@ -2677,8 +2686,8 @@
       <c r="J32" t="s">
         <v>11</v>
       </c>
-      <c r="K32">
-        <v>100</v>
+      <c r="K32" s="2">
+        <v>1</v>
       </c>
       <c r="L32" t="s">
         <v>125</v>
@@ -2699,7 +2708,7 @@
         <v>37</v>
       </c>
       <c r="R32" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="S32" t="s">
         <v>42</v>
@@ -2751,8 +2760,8 @@
       <c r="J33" t="s">
         <v>11</v>
       </c>
-      <c r="K33">
-        <v>100</v>
+      <c r="K33" s="2">
+        <v>1</v>
       </c>
       <c r="L33" t="s">
         <v>125</v>
@@ -2773,7 +2782,7 @@
         <v>37</v>
       </c>
       <c r="R33" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="S33" t="s">
         <v>42</v>
@@ -2825,11 +2834,11 @@
       <c r="J34" t="s">
         <v>11</v>
       </c>
-      <c r="K34">
-        <v>50</v>
+      <c r="K34" s="2">
+        <v>1</v>
       </c>
       <c r="L34" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="M34" t="s">
         <v>11</v>
@@ -2847,10 +2856,10 @@
         <v>37</v>
       </c>
       <c r="R34" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="S34" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T34" t="s">
         <v>11</v>
@@ -2899,7 +2908,7 @@
       <c r="J35" t="s">
         <v>11</v>
       </c>
-      <c r="K35">
+      <c r="K35" s="2">
         <v>0</v>
       </c>
       <c r="L35" t="s">
@@ -2921,7 +2930,7 @@
         <v>37</v>
       </c>
       <c r="R35" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="S35" t="s">
         <v>11</v>
@@ -2973,8 +2982,8 @@
       <c r="J36" t="s">
         <v>11</v>
       </c>
-      <c r="K36">
-        <v>100</v>
+      <c r="K36" s="2">
+        <v>1</v>
       </c>
       <c r="L36" t="s">
         <v>125</v>
@@ -2995,7 +3004,7 @@
         <v>37</v>
       </c>
       <c r="R36" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="S36" t="s">
         <v>42</v>
@@ -3047,8 +3056,8 @@
       <c r="J37" t="s">
         <v>11</v>
       </c>
-      <c r="K37">
-        <v>100</v>
+      <c r="K37" s="2">
+        <v>1</v>
       </c>
       <c r="L37" t="s">
         <v>125</v>
@@ -3069,7 +3078,7 @@
         <v>37</v>
       </c>
       <c r="R37" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="S37" t="s">
         <v>42</v>
@@ -3121,7 +3130,7 @@
       <c r="J38" t="s">
         <v>11</v>
       </c>
-      <c r="K38">
+      <c r="K38" s="2">
         <v>0</v>
       </c>
       <c r="L38" t="s">
@@ -3186,20 +3195,20 @@
       <c r="G39" t="s">
         <v>11</v>
       </c>
-      <c r="H39">
+      <c r="H39" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I39">
+      <c r="I39" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J39" t="s">
         <v>11</v>
       </c>
-      <c r="K39">
-        <v>70</v>
+      <c r="K39" s="2">
+        <v>1</v>
       </c>
       <c r="L39" t="s">
-        <v>11</v>
+        <v>125</v>
       </c>
       <c r="M39" t="s">
         <v>11</v>
@@ -3217,10 +3226,10 @@
         <v>37</v>
       </c>
       <c r="R39" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="S39" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T39" t="s">
         <v>11</v>
@@ -3260,20 +3269,20 @@
       <c r="G40" t="s">
         <v>11</v>
       </c>
-      <c r="H40">
+      <c r="H40" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I40">
+      <c r="I40" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J40" t="s">
         <v>11</v>
       </c>
-      <c r="K40">
-        <v>0</v>
+      <c r="K40" s="2">
+        <v>1</v>
       </c>
       <c r="L40" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M40" t="s">
         <v>11</v>
@@ -3291,10 +3300,10 @@
         <v>37</v>
       </c>
       <c r="R40" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S40" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T40" t="s">
         <v>11</v>
@@ -3334,20 +3343,20 @@
       <c r="G41" t="s">
         <v>11</v>
       </c>
-      <c r="H41">
+      <c r="H41" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I41">
+      <c r="I41" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J41" t="s">
         <v>11</v>
       </c>
-      <c r="K41">
-        <v>50</v>
+      <c r="K41" s="2">
+        <v>1</v>
       </c>
       <c r="L41" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="M41" t="s">
         <v>11</v>
@@ -3365,10 +3374,10 @@
         <v>37</v>
       </c>
       <c r="R41" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="S41" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T41" t="s">
         <v>11</v>
@@ -3408,20 +3417,20 @@
       <c r="G42" t="s">
         <v>11</v>
       </c>
-      <c r="H42">
+      <c r="H42" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I42">
+      <c r="I42" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J42" t="s">
         <v>11</v>
       </c>
-      <c r="K42">
-        <v>50</v>
+      <c r="K42" s="2">
+        <v>1</v>
       </c>
       <c r="L42" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="M42" t="s">
         <v>11</v>
@@ -3439,10 +3448,10 @@
         <v>37</v>
       </c>
       <c r="R42" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="S42" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T42" t="s">
         <v>11</v>
@@ -3482,20 +3491,20 @@
       <c r="G43" t="s">
         <v>11</v>
       </c>
-      <c r="H43">
+      <c r="H43" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I43">
+      <c r="I43" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J43" t="s">
         <v>11</v>
       </c>
-      <c r="K43">
-        <v>50</v>
+      <c r="K43" s="2">
+        <v>1</v>
       </c>
       <c r="L43" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="M43" t="s">
         <v>11</v>
@@ -3513,10 +3522,10 @@
         <v>37</v>
       </c>
       <c r="R43" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="S43" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T43" t="s">
         <v>11</v>
@@ -3556,20 +3565,20 @@
       <c r="G44" t="s">
         <v>11</v>
       </c>
-      <c r="H44">
+      <c r="H44" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I44">
+      <c r="I44" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J44" t="s">
         <v>11</v>
       </c>
-      <c r="K44">
-        <v>0</v>
+      <c r="K44" s="2">
+        <v>1</v>
       </c>
       <c r="L44" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M44" t="s">
         <v>11</v>
@@ -3587,10 +3596,10 @@
         <v>37</v>
       </c>
       <c r="R44" t="s">
-        <v>11</v>
+        <v>157</v>
       </c>
       <c r="S44" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="T44" t="s">
         <v>11</v>
@@ -3630,17 +3639,17 @@
       <c r="G45" t="s">
         <v>11</v>
       </c>
-      <c r="H45">
+      <c r="H45" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I45">
+      <c r="I45" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J45" t="s">
         <v>11</v>
       </c>
-      <c r="K45">
-        <v>100</v>
+      <c r="K45" s="2">
+        <v>1</v>
       </c>
       <c r="L45" t="s">
         <v>125</v>
@@ -3661,7 +3670,7 @@
         <v>37</v>
       </c>
       <c r="R45" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="S45" t="s">
         <v>42</v>
@@ -3704,16 +3713,16 @@
       <c r="G46" t="s">
         <v>11</v>
       </c>
-      <c r="H46">
+      <c r="H46" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I46">
+      <c r="I46" s="1">
         <v>46150.708333333299</v>
       </c>
       <c r="J46" t="s">
         <v>11</v>
       </c>
-      <c r="K46">
+      <c r="K46" s="2">
         <v>0</v>
       </c>
       <c r="L46" t="s">
@@ -3778,17 +3787,17 @@
       <c r="G47" t="s">
         <v>11</v>
       </c>
-      <c r="H47">
+      <c r="H47" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I47">
+      <c r="I47" s="1">
         <v>46148.708333333299</v>
       </c>
       <c r="J47" t="s">
         <v>11</v>
       </c>
-      <c r="K47">
-        <v>100</v>
+      <c r="K47" s="2">
+        <v>1</v>
       </c>
       <c r="L47" t="s">
         <v>11</v>
@@ -3852,17 +3861,17 @@
       <c r="G48" t="s">
         <v>11</v>
       </c>
-      <c r="H48">
+      <c r="H48" s="1">
         <v>46148.375</v>
       </c>
-      <c r="I48">
+      <c r="I48" s="1">
         <v>46148.708333333299</v>
       </c>
       <c r="J48" t="s">
         <v>11</v>
       </c>
-      <c r="K48">
-        <v>100</v>
+      <c r="K48" s="2">
+        <v>1</v>
       </c>
       <c r="L48" t="s">
         <v>125</v>
@@ -3883,7 +3892,7 @@
         <v>37</v>
       </c>
       <c r="R48" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="S48" t="s">
         <v>42</v>
@@ -3935,8 +3944,8 @@
       <c r="J49" t="s">
         <v>11</v>
       </c>
-      <c r="K49">
-        <v>100</v>
+      <c r="K49" s="2">
+        <v>1</v>
       </c>
       <c r="L49" t="s">
         <v>125</v>
@@ -3957,7 +3966,7 @@
         <v>37</v>
       </c>
       <c r="R49" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="S49" t="s">
         <v>42</v>
@@ -4009,8 +4018,8 @@
       <c r="J50" t="s">
         <v>11</v>
       </c>
-      <c r="K50">
-        <v>100</v>
+      <c r="K50" s="2">
+        <v>1</v>
       </c>
       <c r="L50" t="s">
         <v>125</v>
@@ -4031,7 +4040,7 @@
         <v>37</v>
       </c>
       <c r="R50" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="S50" t="s">
         <v>42</v>
@@ -4083,8 +4092,8 @@
       <c r="J51" t="s">
         <v>11</v>
       </c>
-      <c r="K51">
-        <v>100</v>
+      <c r="K51" s="2">
+        <v>1</v>
       </c>
       <c r="L51" t="s">
         <v>125</v>
@@ -4105,7 +4114,7 @@
         <v>37</v>
       </c>
       <c r="R51" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="S51" t="s">
         <v>42</v>
@@ -4129,7 +4138,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:X10 A23:Q23 A11:K11 M11:Q11 A12:K12 M12:Q12 A13:K13 M13:Q13 A14:K14 M14:Q14 A15:K15 M15:Q15 A16:K16 M16:Q16 A17:K17 M17:Q17 A18:K18 M18:Q18 A19:K19 M19:Q19 A20:K20 M20:Q20 A21:K21 M21:Q21 A22:K22 M22:Q22 A28:Q28 A24:K24 M24:Q24 A25:K25 M25:Q25 A26:K26 M26:Q26 A27:K27 M27:Q27 A39:Q39 A29:K29 M29:Q29 A30:K30 M30:Q30 A31:K31 M31:Q31 A32:K32 M32:Q32 A33:K33 M33:Q33 A34:K34 M34:Q34 A35:K35 M35:Q35 A36:K36 M36:Q36 A37:K37 M37:Q37 A38:K38 M38:X38 A47:X47 A40:K40 M40:Q40 A41:K41 M41:Q41 A42:K42 M42:Q42 A43:K43 M43:Q43 A44:K44 M44:X44 A45:K45 M45:Q45 A46:K46 M46:X46 A51:K51 A48:K48 M48:Q48 A49:K49 M49:Q49 A50:K50 M50:Q50 M51:Q51 S11:X11 S12:X12 S13:X13 S14:X14 S15:X15 S16:X16 S17:X17 S18:X18 S19:X19 S20:X20 S21:X21 S22:X22 S23:X23 S24:X24 S25:X25 S26:X26 S27:X27 S28:X28 S29:X29 S30:X30 S31:X31 S32:X32 S33:X33 S34:X34 S35:X35 S36:X36 S37:X37 S39:X39 S40:X40 S41:X41 S42:X42 S43:X43 S45:X45 S48:X48 S49:X49 S50:X50 S51:X51" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:X5 A23:J23 A11:J11 M11:Q11 A12:J12 M12:Q12 A13:J13 M13:Q13 A14:J14 M14:Q14 A15:J15 M15:Q15 A16:J16 M16:Q16 A17:J17 M17:Q17 A18:J18 M18:Q18 A19:J19 M19:Q19 A20:J20 M20:Q20 A21:J21 M21:Q21 A22:J22 M22:Q22 A28:J28 A24:J24 M24:Q24 A25:J25 M25:Q25 A26:J26 M26:Q26 A27:J27 M27:Q27 A39:J39 A29:J29 M29:Q29 A30:J30 M30:Q30 A31:J31 M31:Q31 A32:J32 M32:Q32 A33:J33 M33:Q33 A34:J34 M34:Q34 A35:K35 M35:Q35 A36:J36 M36:Q36 A37:J37 M37:Q37 A38:K38 M38:X38 A47:J47 A40:J40 M40:Q40 A41:J41 M41:Q41 A42:J42 M42:Q42 A43:J43 M43:Q43 A44:J44 M44:Q44 A45:J45 M45:Q45 A46:K46 M46:X46 A51:J51 A48:J48 M48:Q48 A49:J49 M49:Q49 A50:J50 M50:Q50 M51:Q51 S11:X11 S12:X12 S13:X13 S14:X14 S15:X15 S16:X16 T17:X17 S18:X18 S19:X19 S20:X20 S21:X21 S22:X22 T23:X23 S24:X24 S25:X25 S26:X26 S27:X27 T28:X28 S29:X29 S30:X30 S31:X31 S32:X32 S33:X33 T34:X34 S35:X35 S36:X36 S37:X37 T39:X39 T40:X40 T41:X41 T42:X42 T43:X43 S45:X45 S48:X48 S49:X49 S50:X50 S51:X51 A7:X9 A6 C6:X6 M23:Q23 M28:Q28 M39:Q39 T44:X44 A10:J10 M10:R10 L47:X47 T10:X10" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>